<commit_message>
Add date-range Statement of Account; regenerate sample reports
- Spec 3.5: GET /reports/soa/:id accepts dateFrom/dateTo and returns the
  period statement (opening balance, the period's ledger entries, totals,
  closing balance) from the same ledger computation as /reports/ledger.
  The PDF/XLSX export prints that statement; the desktop statement view
  has From/To pickers (default: this month).
- Ledger lines now cite receipt and invoice numbers and the payment
  method ("OR-5001 · Cash payment applied to DEMO-INV-0065") instead of
  internal row IDs.
- reports-samples/: 18 PDF/XLSX files exported from the running system
  against the seeded demo data (monthly and daily collection, AR aging,
  period SOA, ledger, remittance, collector performance and assignments,
  billing vs collection, revenue by plan, master list, reversals/voids,
  voided receipts, user activity, audit trail) (spec D6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports-samples/ar-aging-report.xlsx
+++ b/reports-samples/ar-aging-report.xlsx
@@ -25,7 +25,7 @@
     <t>current</t>
   </si>
   <si>
-    <t>35751.50</t>
+    <t>30254.50</t>
   </si>
   <si>
     <t>1-30</t>
@@ -49,7 +49,7 @@
     <t>90+</t>
   </si>
   <si>
-    <t>4447.00</t>
+    <t>2448.00</t>
   </si>
 </sst>
 </file>
@@ -459,7 +459,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
@@ -503,7 +503,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>12</v>

</xml_diff>